<commit_message>
Fix instruction row 7 text clipping on template Instructions sheet
Longer step 7 text was overflowing the fixed 42px row height. Now
dynamically sets height to 58px for text over 150 characters.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template_NEW_With_Subtotals.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template_NEW_With_Subtotals.xlsx
@@ -633,7 +633,7 @@
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>2.</t>
@@ -705,7 +705,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="58" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>7.</t>

</xml_diff>